<commit_message>
docs: complete implementation specifications and agent coordination baseline
</commit_message>
<xml_diff>
--- a/docs/templates/期初盘点模板.xlsx
+++ b/docs/templates/期初盘点模板.xlsx
@@ -3454,8 +3454,8 @@
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="每个SKU一个唯一编号，宝可梦PK-前缀，符文战场RB-前缀；不同单位分别编号。" errorTitle="请检查输入" error="编号已重复。" sqref="A2:A5001">
       <formula1>COUNTIF($A$2:$A$5001,A2)=1</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="选择卡牌或周边。" errorTitle="请检查输入" error="请选择卡牌或周边。" sqref="C2:C5001">
-      <formula1>"卡牌,周边"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="选择补充包、周边或礼盒/套装/预组。" errorTitle="请检查输入" error="请选择补充包、周边或礼盒/套装/预组。" sqref="C2:C5001">
+      <formula1>"补充包,周边,礼盒/套装/预组"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="肥包、瘦包或留空；包规格在J列自由填写。" errorTitle="请检查输入" error="请选择肥包、瘦包或留空。" sqref="K2:K5001">
       <formula1>"肥包,瘦包"</formula1>

</xml_diff>

<commit_message>
docs: simplify product classification and queue final stage 1 fixes
</commit_message>
<xml_diff>
--- a/docs/templates/期初盘点模板.xlsx
+++ b/docs/templates/期初盘点模板.xlsx
@@ -3454,8 +3454,8 @@
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="每个SKU一个唯一编号，宝可梦PK-前缀，符文战场RB-前缀；不同单位分别编号。" errorTitle="请检查输入" error="编号已重复。" sqref="A2:A5001">
       <formula1>COUNTIF($A$2:$A$5001,A2)=1</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="选择补充包、周边或礼盒/套装/预组。" errorTitle="请检查输入" error="请选择补充包、周边或礼盒/套装/预组。" sqref="C2:C5001">
-      <formula1>"补充包,周边,礼盒/套装/预组"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="选择补充包、周边或礼盒·预组。" errorTitle="请检查输入" error="请选择补充包、周边或礼盒·预组。" sqref="C2:C5001">
+      <formula1>"补充包,周边,礼盒·预组"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="肥包、瘦包或留空；包规格在J列自由填写。" errorTitle="请检查输入" error="请选择肥包、瘦包或留空。" sqref="K2:K5001">
       <formula1>"肥包,瘦包"</formula1>

</xml_diff>

<commit_message>
docs: add optional inner box specification and update opening template
</commit_message>
<xml_diff>
--- a/docs/templates/期初盘点模板.xlsx
+++ b/docs/templates/期初盘点模板.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>商品内部编号</t>
   </si>
@@ -85,6 +85,9 @@
   </si>
   <si>
     <t>备注</t>
+  </si>
+  <si>
+    <t>盒规格</t>
   </si>
 </sst>
 </file>
@@ -185,7 +188,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N201"/>
+  <dimension ref="A1:O201"/>
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1" style="13"/>
@@ -198,10 +201,11 @@
     <col min="8" max="8" width="18" customWidth="1" style="13"/>
     <col min="9" max="9" width="22" customWidth="1" style="13"/>
     <col min="10" max="10" width="22" customWidth="1" style="13"/>
-    <col min="11" max="11" width="12" customWidth="1" style="13"/>
+    <col min="11" max="11" width="22" customWidth="1" style="13"/>
     <col min="12" max="12" width="12" customWidth="1" style="13"/>
-    <col min="13" max="13" width="22" customWidth="1" style="13"/>
-    <col min="14" max="14" width="26" customWidth="1" style="13"/>
+    <col min="13" max="13" width="12" customWidth="1" style="13"/>
+    <col min="14" max="14" width="22" customWidth="1" style="13"/>
+    <col min="15" max="15" width="26" customWidth="1" style="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -233,18 +237,21 @@
         <v>8</v>
       </c>
       <c r="J1" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="15" t="s">
+      <c r="L1" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="15" t="s">
+      <c r="M1" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="15" t="s">
+      <c r="N1" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="15" t="s">
+      <c r="O1" s="15" t="s">
         <v>13</v>
       </c>
     </row>
@@ -263,6 +270,7 @@
       <c r="L2" s="13"/>
       <c r="M2" s="13"/>
       <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
     </row>
     <row r="3">
       <c r="A3" s="13"/>
@@ -279,6 +287,7 @@
       <c r="L3" s="13"/>
       <c r="M3" s="13"/>
       <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
     </row>
     <row r="4">
       <c r="A4" s="13"/>
@@ -295,6 +304,7 @@
       <c r="L4" s="13"/>
       <c r="M4" s="13"/>
       <c r="N4" s="13"/>
+      <c r="O4" s="13"/>
     </row>
     <row r="5">
       <c r="A5" s="13"/>
@@ -311,6 +321,7 @@
       <c r="L5" s="13"/>
       <c r="M5" s="13"/>
       <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
     </row>
     <row r="6">
       <c r="A6" s="13"/>
@@ -327,6 +338,7 @@
       <c r="L6" s="13"/>
       <c r="M6" s="13"/>
       <c r="N6" s="13"/>
+      <c r="O6" s="13"/>
     </row>
     <row r="7">
       <c r="A7" s="13"/>
@@ -343,6 +355,7 @@
       <c r="L7" s="13"/>
       <c r="M7" s="13"/>
       <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
     </row>
     <row r="8">
       <c r="A8" s="13"/>
@@ -359,6 +372,7 @@
       <c r="L8" s="13"/>
       <c r="M8" s="13"/>
       <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
     </row>
     <row r="9">
       <c r="A9" s="13"/>
@@ -375,6 +389,7 @@
       <c r="L9" s="13"/>
       <c r="M9" s="13"/>
       <c r="N9" s="13"/>
+      <c r="O9" s="13"/>
     </row>
     <row r="10">
       <c r="A10" s="13"/>
@@ -391,6 +406,7 @@
       <c r="L10" s="13"/>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
     </row>
     <row r="11">
       <c r="A11" s="13"/>
@@ -407,6 +423,7 @@
       <c r="L11" s="13"/>
       <c r="M11" s="13"/>
       <c r="N11" s="13"/>
+      <c r="O11" s="13"/>
     </row>
     <row r="12">
       <c r="A12" s="13"/>
@@ -423,6 +440,7 @@
       <c r="L12" s="13"/>
       <c r="M12" s="13"/>
       <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
     </row>
     <row r="13">
       <c r="A13" s="13"/>
@@ -439,6 +457,7 @@
       <c r="L13" s="13"/>
       <c r="M13" s="13"/>
       <c r="N13" s="13"/>
+      <c r="O13" s="13"/>
     </row>
     <row r="14">
       <c r="A14" s="13"/>
@@ -455,6 +474,7 @@
       <c r="L14" s="13"/>
       <c r="M14" s="13"/>
       <c r="N14" s="13"/>
+      <c r="O14" s="13"/>
     </row>
     <row r="15">
       <c r="A15" s="13"/>
@@ -471,6 +491,7 @@
       <c r="L15" s="13"/>
       <c r="M15" s="13"/>
       <c r="N15" s="13"/>
+      <c r="O15" s="13"/>
     </row>
     <row r="16">
       <c r="A16" s="13"/>
@@ -487,6 +508,7 @@
       <c r="L16" s="13"/>
       <c r="M16" s="13"/>
       <c r="N16" s="13"/>
+      <c r="O16" s="13"/>
     </row>
     <row r="17">
       <c r="A17" s="13"/>
@@ -503,6 +525,7 @@
       <c r="L17" s="13"/>
       <c r="M17" s="13"/>
       <c r="N17" s="13"/>
+      <c r="O17" s="13"/>
     </row>
     <row r="18">
       <c r="A18" s="13"/>
@@ -519,6 +542,7 @@
       <c r="L18" s="13"/>
       <c r="M18" s="13"/>
       <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
     </row>
     <row r="19">
       <c r="A19" s="13"/>
@@ -535,6 +559,7 @@
       <c r="L19" s="13"/>
       <c r="M19" s="13"/>
       <c r="N19" s="13"/>
+      <c r="O19" s="13"/>
     </row>
     <row r="20">
       <c r="A20" s="13"/>
@@ -551,6 +576,7 @@
       <c r="L20" s="13"/>
       <c r="M20" s="13"/>
       <c r="N20" s="13"/>
+      <c r="O20" s="13"/>
     </row>
     <row r="21">
       <c r="A21" s="13"/>
@@ -567,6 +593,7 @@
       <c r="L21" s="13"/>
       <c r="M21" s="13"/>
       <c r="N21" s="13"/>
+      <c r="O21" s="13"/>
     </row>
     <row r="22">
       <c r="A22" s="13"/>
@@ -583,6 +610,7 @@
       <c r="L22" s="13"/>
       <c r="M22" s="13"/>
       <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
     </row>
     <row r="23">
       <c r="A23" s="13"/>
@@ -599,6 +627,7 @@
       <c r="L23" s="13"/>
       <c r="M23" s="13"/>
       <c r="N23" s="13"/>
+      <c r="O23" s="13"/>
     </row>
     <row r="24">
       <c r="A24" s="13"/>
@@ -615,6 +644,7 @@
       <c r="L24" s="13"/>
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
+      <c r="O24" s="13"/>
     </row>
     <row r="25">
       <c r="A25" s="13"/>
@@ -631,6 +661,7 @@
       <c r="L25" s="13"/>
       <c r="M25" s="13"/>
       <c r="N25" s="13"/>
+      <c r="O25" s="13"/>
     </row>
     <row r="26">
       <c r="A26" s="13"/>
@@ -647,6 +678,7 @@
       <c r="L26" s="13"/>
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
+      <c r="O26" s="13"/>
     </row>
     <row r="27">
       <c r="A27" s="13"/>
@@ -663,6 +695,7 @@
       <c r="L27" s="13"/>
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
+      <c r="O27" s="13"/>
     </row>
     <row r="28">
       <c r="A28" s="13"/>
@@ -679,6 +712,7 @@
       <c r="L28" s="13"/>
       <c r="M28" s="13"/>
       <c r="N28" s="13"/>
+      <c r="O28" s="13"/>
     </row>
     <row r="29">
       <c r="A29" s="13"/>
@@ -695,6 +729,7 @@
       <c r="L29" s="13"/>
       <c r="M29" s="13"/>
       <c r="N29" s="13"/>
+      <c r="O29" s="13"/>
     </row>
     <row r="30">
       <c r="A30" s="13"/>
@@ -711,6 +746,7 @@
       <c r="L30" s="13"/>
       <c r="M30" s="13"/>
       <c r="N30" s="13"/>
+      <c r="O30" s="13"/>
     </row>
     <row r="31">
       <c r="A31" s="13"/>
@@ -727,6 +763,7 @@
       <c r="L31" s="13"/>
       <c r="M31" s="13"/>
       <c r="N31" s="13"/>
+      <c r="O31" s="13"/>
     </row>
     <row r="32">
       <c r="A32" s="13"/>
@@ -743,6 +780,7 @@
       <c r="L32" s="13"/>
       <c r="M32" s="13"/>
       <c r="N32" s="13"/>
+      <c r="O32" s="13"/>
     </row>
     <row r="33">
       <c r="A33" s="13"/>
@@ -759,6 +797,7 @@
       <c r="L33" s="13"/>
       <c r="M33" s="13"/>
       <c r="N33" s="13"/>
+      <c r="O33" s="13"/>
     </row>
     <row r="34">
       <c r="A34" s="13"/>
@@ -775,6 +814,7 @@
       <c r="L34" s="13"/>
       <c r="M34" s="13"/>
       <c r="N34" s="13"/>
+      <c r="O34" s="13"/>
     </row>
     <row r="35">
       <c r="A35" s="13"/>
@@ -791,6 +831,7 @@
       <c r="L35" s="13"/>
       <c r="M35" s="13"/>
       <c r="N35" s="13"/>
+      <c r="O35" s="13"/>
     </row>
     <row r="36">
       <c r="A36" s="13"/>
@@ -807,6 +848,7 @@
       <c r="L36" s="13"/>
       <c r="M36" s="13"/>
       <c r="N36" s="13"/>
+      <c r="O36" s="13"/>
     </row>
     <row r="37">
       <c r="A37" s="13"/>
@@ -823,6 +865,7 @@
       <c r="L37" s="13"/>
       <c r="M37" s="13"/>
       <c r="N37" s="13"/>
+      <c r="O37" s="13"/>
     </row>
     <row r="38">
       <c r="A38" s="13"/>
@@ -839,6 +882,7 @@
       <c r="L38" s="13"/>
       <c r="M38" s="13"/>
       <c r="N38" s="13"/>
+      <c r="O38" s="13"/>
     </row>
     <row r="39">
       <c r="A39" s="13"/>
@@ -855,6 +899,7 @@
       <c r="L39" s="13"/>
       <c r="M39" s="13"/>
       <c r="N39" s="13"/>
+      <c r="O39" s="13"/>
     </row>
     <row r="40">
       <c r="A40" s="13"/>
@@ -871,6 +916,7 @@
       <c r="L40" s="13"/>
       <c r="M40" s="13"/>
       <c r="N40" s="13"/>
+      <c r="O40" s="13"/>
     </row>
     <row r="41">
       <c r="A41" s="13"/>
@@ -887,6 +933,7 @@
       <c r="L41" s="13"/>
       <c r="M41" s="13"/>
       <c r="N41" s="13"/>
+      <c r="O41" s="13"/>
     </row>
     <row r="42">
       <c r="A42" s="13"/>
@@ -903,6 +950,7 @@
       <c r="L42" s="13"/>
       <c r="M42" s="13"/>
       <c r="N42" s="13"/>
+      <c r="O42" s="13"/>
     </row>
     <row r="43">
       <c r="A43" s="13"/>
@@ -919,6 +967,7 @@
       <c r="L43" s="13"/>
       <c r="M43" s="13"/>
       <c r="N43" s="13"/>
+      <c r="O43" s="13"/>
     </row>
     <row r="44">
       <c r="A44" s="13"/>
@@ -935,6 +984,7 @@
       <c r="L44" s="13"/>
       <c r="M44" s="13"/>
       <c r="N44" s="13"/>
+      <c r="O44" s="13"/>
     </row>
     <row r="45">
       <c r="A45" s="13"/>
@@ -951,6 +1001,7 @@
       <c r="L45" s="13"/>
       <c r="M45" s="13"/>
       <c r="N45" s="13"/>
+      <c r="O45" s="13"/>
     </row>
     <row r="46">
       <c r="A46" s="13"/>
@@ -967,6 +1018,7 @@
       <c r="L46" s="13"/>
       <c r="M46" s="13"/>
       <c r="N46" s="13"/>
+      <c r="O46" s="13"/>
     </row>
     <row r="47">
       <c r="A47" s="13"/>
@@ -983,6 +1035,7 @@
       <c r="L47" s="13"/>
       <c r="M47" s="13"/>
       <c r="N47" s="13"/>
+      <c r="O47" s="13"/>
     </row>
     <row r="48">
       <c r="A48" s="13"/>
@@ -999,6 +1052,7 @@
       <c r="L48" s="13"/>
       <c r="M48" s="13"/>
       <c r="N48" s="13"/>
+      <c r="O48" s="13"/>
     </row>
     <row r="49">
       <c r="A49" s="13"/>
@@ -1015,6 +1069,7 @@
       <c r="L49" s="13"/>
       <c r="M49" s="13"/>
       <c r="N49" s="13"/>
+      <c r="O49" s="13"/>
     </row>
     <row r="50">
       <c r="A50" s="13"/>
@@ -1031,6 +1086,7 @@
       <c r="L50" s="13"/>
       <c r="M50" s="13"/>
       <c r="N50" s="13"/>
+      <c r="O50" s="13"/>
     </row>
     <row r="51">
       <c r="A51" s="13"/>
@@ -1047,6 +1103,7 @@
       <c r="L51" s="13"/>
       <c r="M51" s="13"/>
       <c r="N51" s="13"/>
+      <c r="O51" s="13"/>
     </row>
     <row r="52">
       <c r="A52" s="13"/>
@@ -1063,6 +1120,7 @@
       <c r="L52" s="13"/>
       <c r="M52" s="13"/>
       <c r="N52" s="13"/>
+      <c r="O52" s="13"/>
     </row>
     <row r="53">
       <c r="A53" s="13"/>
@@ -1079,6 +1137,7 @@
       <c r="L53" s="13"/>
       <c r="M53" s="13"/>
       <c r="N53" s="13"/>
+      <c r="O53" s="13"/>
     </row>
     <row r="54">
       <c r="A54" s="13"/>
@@ -1095,6 +1154,7 @@
       <c r="L54" s="13"/>
       <c r="M54" s="13"/>
       <c r="N54" s="13"/>
+      <c r="O54" s="13"/>
     </row>
     <row r="55">
       <c r="A55" s="13"/>
@@ -1111,6 +1171,7 @@
       <c r="L55" s="13"/>
       <c r="M55" s="13"/>
       <c r="N55" s="13"/>
+      <c r="O55" s="13"/>
     </row>
     <row r="56">
       <c r="A56" s="13"/>
@@ -1127,6 +1188,7 @@
       <c r="L56" s="13"/>
       <c r="M56" s="13"/>
       <c r="N56" s="13"/>
+      <c r="O56" s="13"/>
     </row>
     <row r="57">
       <c r="A57" s="13"/>
@@ -1143,6 +1205,7 @@
       <c r="L57" s="13"/>
       <c r="M57" s="13"/>
       <c r="N57" s="13"/>
+      <c r="O57" s="13"/>
     </row>
     <row r="58">
       <c r="A58" s="13"/>
@@ -1159,6 +1222,7 @@
       <c r="L58" s="13"/>
       <c r="M58" s="13"/>
       <c r="N58" s="13"/>
+      <c r="O58" s="13"/>
     </row>
     <row r="59">
       <c r="A59" s="13"/>
@@ -1175,6 +1239,7 @@
       <c r="L59" s="13"/>
       <c r="M59" s="13"/>
       <c r="N59" s="13"/>
+      <c r="O59" s="13"/>
     </row>
     <row r="60">
       <c r="A60" s="13"/>
@@ -1191,6 +1256,7 @@
       <c r="L60" s="13"/>
       <c r="M60" s="13"/>
       <c r="N60" s="13"/>
+      <c r="O60" s="13"/>
     </row>
     <row r="61">
       <c r="A61" s="13"/>
@@ -1207,6 +1273,7 @@
       <c r="L61" s="13"/>
       <c r="M61" s="13"/>
       <c r="N61" s="13"/>
+      <c r="O61" s="13"/>
     </row>
     <row r="62">
       <c r="A62" s="13"/>
@@ -1223,6 +1290,7 @@
       <c r="L62" s="13"/>
       <c r="M62" s="13"/>
       <c r="N62" s="13"/>
+      <c r="O62" s="13"/>
     </row>
     <row r="63">
       <c r="A63" s="13"/>
@@ -1239,6 +1307,7 @@
       <c r="L63" s="13"/>
       <c r="M63" s="13"/>
       <c r="N63" s="13"/>
+      <c r="O63" s="13"/>
     </row>
     <row r="64">
       <c r="A64" s="13"/>
@@ -1255,6 +1324,7 @@
       <c r="L64" s="13"/>
       <c r="M64" s="13"/>
       <c r="N64" s="13"/>
+      <c r="O64" s="13"/>
     </row>
     <row r="65">
       <c r="A65" s="13"/>
@@ -1271,6 +1341,7 @@
       <c r="L65" s="13"/>
       <c r="M65" s="13"/>
       <c r="N65" s="13"/>
+      <c r="O65" s="13"/>
     </row>
     <row r="66">
       <c r="A66" s="13"/>
@@ -1287,6 +1358,7 @@
       <c r="L66" s="13"/>
       <c r="M66" s="13"/>
       <c r="N66" s="13"/>
+      <c r="O66" s="13"/>
     </row>
     <row r="67">
       <c r="A67" s="13"/>
@@ -1303,6 +1375,7 @@
       <c r="L67" s="13"/>
       <c r="M67" s="13"/>
       <c r="N67" s="13"/>
+      <c r="O67" s="13"/>
     </row>
     <row r="68">
       <c r="A68" s="13"/>
@@ -1319,6 +1392,7 @@
       <c r="L68" s="13"/>
       <c r="M68" s="13"/>
       <c r="N68" s="13"/>
+      <c r="O68" s="13"/>
     </row>
     <row r="69">
       <c r="A69" s="13"/>
@@ -1335,6 +1409,7 @@
       <c r="L69" s="13"/>
       <c r="M69" s="13"/>
       <c r="N69" s="13"/>
+      <c r="O69" s="13"/>
     </row>
     <row r="70">
       <c r="A70" s="13"/>
@@ -1351,6 +1426,7 @@
       <c r="L70" s="13"/>
       <c r="M70" s="13"/>
       <c r="N70" s="13"/>
+      <c r="O70" s="13"/>
     </row>
     <row r="71">
       <c r="A71" s="13"/>
@@ -1367,6 +1443,7 @@
       <c r="L71" s="13"/>
       <c r="M71" s="13"/>
       <c r="N71" s="13"/>
+      <c r="O71" s="13"/>
     </row>
     <row r="72">
       <c r="A72" s="13"/>
@@ -1383,6 +1460,7 @@
       <c r="L72" s="13"/>
       <c r="M72" s="13"/>
       <c r="N72" s="13"/>
+      <c r="O72" s="13"/>
     </row>
     <row r="73">
       <c r="A73" s="13"/>
@@ -1399,6 +1477,7 @@
       <c r="L73" s="13"/>
       <c r="M73" s="13"/>
       <c r="N73" s="13"/>
+      <c r="O73" s="13"/>
     </row>
     <row r="74">
       <c r="A74" s="13"/>
@@ -1415,6 +1494,7 @@
       <c r="L74" s="13"/>
       <c r="M74" s="13"/>
       <c r="N74" s="13"/>
+      <c r="O74" s="13"/>
     </row>
     <row r="75">
       <c r="A75" s="13"/>
@@ -1431,6 +1511,7 @@
       <c r="L75" s="13"/>
       <c r="M75" s="13"/>
       <c r="N75" s="13"/>
+      <c r="O75" s="13"/>
     </row>
     <row r="76">
       <c r="A76" s="13"/>
@@ -1447,6 +1528,7 @@
       <c r="L76" s="13"/>
       <c r="M76" s="13"/>
       <c r="N76" s="13"/>
+      <c r="O76" s="13"/>
     </row>
     <row r="77">
       <c r="A77" s="13"/>
@@ -1463,6 +1545,7 @@
       <c r="L77" s="13"/>
       <c r="M77" s="13"/>
       <c r="N77" s="13"/>
+      <c r="O77" s="13"/>
     </row>
     <row r="78">
       <c r="A78" s="13"/>
@@ -1479,6 +1562,7 @@
       <c r="L78" s="13"/>
       <c r="M78" s="13"/>
       <c r="N78" s="13"/>
+      <c r="O78" s="13"/>
     </row>
     <row r="79">
       <c r="A79" s="13"/>
@@ -1495,6 +1579,7 @@
       <c r="L79" s="13"/>
       <c r="M79" s="13"/>
       <c r="N79" s="13"/>
+      <c r="O79" s="13"/>
     </row>
     <row r="80">
       <c r="A80" s="13"/>
@@ -1511,6 +1596,7 @@
       <c r="L80" s="13"/>
       <c r="M80" s="13"/>
       <c r="N80" s="13"/>
+      <c r="O80" s="13"/>
     </row>
     <row r="81">
       <c r="A81" s="13"/>
@@ -1527,6 +1613,7 @@
       <c r="L81" s="13"/>
       <c r="M81" s="13"/>
       <c r="N81" s="13"/>
+      <c r="O81" s="13"/>
     </row>
     <row r="82">
       <c r="A82" s="13"/>
@@ -1543,6 +1630,7 @@
       <c r="L82" s="13"/>
       <c r="M82" s="13"/>
       <c r="N82" s="13"/>
+      <c r="O82" s="13"/>
     </row>
     <row r="83">
       <c r="A83" s="13"/>
@@ -1559,6 +1647,7 @@
       <c r="L83" s="13"/>
       <c r="M83" s="13"/>
       <c r="N83" s="13"/>
+      <c r="O83" s="13"/>
     </row>
     <row r="84">
       <c r="A84" s="13"/>
@@ -1575,6 +1664,7 @@
       <c r="L84" s="13"/>
       <c r="M84" s="13"/>
       <c r="N84" s="13"/>
+      <c r="O84" s="13"/>
     </row>
     <row r="85">
       <c r="A85" s="13"/>
@@ -1591,6 +1681,7 @@
       <c r="L85" s="13"/>
       <c r="M85" s="13"/>
       <c r="N85" s="13"/>
+      <c r="O85" s="13"/>
     </row>
     <row r="86">
       <c r="A86" s="13"/>
@@ -1607,6 +1698,7 @@
       <c r="L86" s="13"/>
       <c r="M86" s="13"/>
       <c r="N86" s="13"/>
+      <c r="O86" s="13"/>
     </row>
     <row r="87">
       <c r="A87" s="13"/>
@@ -1623,6 +1715,7 @@
       <c r="L87" s="13"/>
       <c r="M87" s="13"/>
       <c r="N87" s="13"/>
+      <c r="O87" s="13"/>
     </row>
     <row r="88">
       <c r="A88" s="13"/>
@@ -1639,6 +1732,7 @@
       <c r="L88" s="13"/>
       <c r="M88" s="13"/>
       <c r="N88" s="13"/>
+      <c r="O88" s="13"/>
     </row>
     <row r="89">
       <c r="A89" s="13"/>
@@ -1655,6 +1749,7 @@
       <c r="L89" s="13"/>
       <c r="M89" s="13"/>
       <c r="N89" s="13"/>
+      <c r="O89" s="13"/>
     </row>
     <row r="90">
       <c r="A90" s="13"/>
@@ -1671,6 +1766,7 @@
       <c r="L90" s="13"/>
       <c r="M90" s="13"/>
       <c r="N90" s="13"/>
+      <c r="O90" s="13"/>
     </row>
     <row r="91">
       <c r="A91" s="13"/>
@@ -1687,6 +1783,7 @@
       <c r="L91" s="13"/>
       <c r="M91" s="13"/>
       <c r="N91" s="13"/>
+      <c r="O91" s="13"/>
     </row>
     <row r="92">
       <c r="A92" s="13"/>
@@ -1703,6 +1800,7 @@
       <c r="L92" s="13"/>
       <c r="M92" s="13"/>
       <c r="N92" s="13"/>
+      <c r="O92" s="13"/>
     </row>
     <row r="93">
       <c r="A93" s="13"/>
@@ -1719,6 +1817,7 @@
       <c r="L93" s="13"/>
       <c r="M93" s="13"/>
       <c r="N93" s="13"/>
+      <c r="O93" s="13"/>
     </row>
     <row r="94">
       <c r="A94" s="13"/>
@@ -1735,6 +1834,7 @@
       <c r="L94" s="13"/>
       <c r="M94" s="13"/>
       <c r="N94" s="13"/>
+      <c r="O94" s="13"/>
     </row>
     <row r="95">
       <c r="A95" s="13"/>
@@ -1751,6 +1851,7 @@
       <c r="L95" s="13"/>
       <c r="M95" s="13"/>
       <c r="N95" s="13"/>
+      <c r="O95" s="13"/>
     </row>
     <row r="96">
       <c r="A96" s="13"/>
@@ -1767,6 +1868,7 @@
       <c r="L96" s="13"/>
       <c r="M96" s="13"/>
       <c r="N96" s="13"/>
+      <c r="O96" s="13"/>
     </row>
     <row r="97">
       <c r="A97" s="13"/>
@@ -1783,6 +1885,7 @@
       <c r="L97" s="13"/>
       <c r="M97" s="13"/>
       <c r="N97" s="13"/>
+      <c r="O97" s="13"/>
     </row>
     <row r="98">
       <c r="A98" s="13"/>
@@ -1799,6 +1902,7 @@
       <c r="L98" s="13"/>
       <c r="M98" s="13"/>
       <c r="N98" s="13"/>
+      <c r="O98" s="13"/>
     </row>
     <row r="99">
       <c r="A99" s="13"/>
@@ -1815,6 +1919,7 @@
       <c r="L99" s="13"/>
       <c r="M99" s="13"/>
       <c r="N99" s="13"/>
+      <c r="O99" s="13"/>
     </row>
     <row r="100">
       <c r="A100" s="13"/>
@@ -1831,6 +1936,7 @@
       <c r="L100" s="13"/>
       <c r="M100" s="13"/>
       <c r="N100" s="13"/>
+      <c r="O100" s="13"/>
     </row>
     <row r="101">
       <c r="A101" s="13"/>
@@ -1847,6 +1953,7 @@
       <c r="L101" s="13"/>
       <c r="M101" s="13"/>
       <c r="N101" s="13"/>
+      <c r="O101" s="13"/>
     </row>
     <row r="102">
       <c r="A102" s="13"/>
@@ -1863,6 +1970,7 @@
       <c r="L102" s="13"/>
       <c r="M102" s="13"/>
       <c r="N102" s="13"/>
+      <c r="O102" s="13"/>
     </row>
     <row r="103">
       <c r="A103" s="13"/>
@@ -1879,6 +1987,7 @@
       <c r="L103" s="13"/>
       <c r="M103" s="13"/>
       <c r="N103" s="13"/>
+      <c r="O103" s="13"/>
     </row>
     <row r="104">
       <c r="A104" s="13"/>
@@ -1895,6 +2004,7 @@
       <c r="L104" s="13"/>
       <c r="M104" s="13"/>
       <c r="N104" s="13"/>
+      <c r="O104" s="13"/>
     </row>
     <row r="105">
       <c r="A105" s="13"/>
@@ -1911,6 +2021,7 @@
       <c r="L105" s="13"/>
       <c r="M105" s="13"/>
       <c r="N105" s="13"/>
+      <c r="O105" s="13"/>
     </row>
     <row r="106">
       <c r="A106" s="13"/>
@@ -1927,6 +2038,7 @@
       <c r="L106" s="13"/>
       <c r="M106" s="13"/>
       <c r="N106" s="13"/>
+      <c r="O106" s="13"/>
     </row>
     <row r="107">
       <c r="A107" s="13"/>
@@ -1943,6 +2055,7 @@
       <c r="L107" s="13"/>
       <c r="M107" s="13"/>
       <c r="N107" s="13"/>
+      <c r="O107" s="13"/>
     </row>
     <row r="108">
       <c r="A108" s="13"/>
@@ -1959,6 +2072,7 @@
       <c r="L108" s="13"/>
       <c r="M108" s="13"/>
       <c r="N108" s="13"/>
+      <c r="O108" s="13"/>
     </row>
     <row r="109">
       <c r="A109" s="13"/>
@@ -1975,6 +2089,7 @@
       <c r="L109" s="13"/>
       <c r="M109" s="13"/>
       <c r="N109" s="13"/>
+      <c r="O109" s="13"/>
     </row>
     <row r="110">
       <c r="A110" s="13"/>
@@ -1991,6 +2106,7 @@
       <c r="L110" s="13"/>
       <c r="M110" s="13"/>
       <c r="N110" s="13"/>
+      <c r="O110" s="13"/>
     </row>
     <row r="111">
       <c r="A111" s="13"/>
@@ -2007,6 +2123,7 @@
       <c r="L111" s="13"/>
       <c r="M111" s="13"/>
       <c r="N111" s="13"/>
+      <c r="O111" s="13"/>
     </row>
     <row r="112">
       <c r="A112" s="13"/>
@@ -2023,6 +2140,7 @@
       <c r="L112" s="13"/>
       <c r="M112" s="13"/>
       <c r="N112" s="13"/>
+      <c r="O112" s="13"/>
     </row>
     <row r="113">
       <c r="A113" s="13"/>
@@ -2039,6 +2157,7 @@
       <c r="L113" s="13"/>
       <c r="M113" s="13"/>
       <c r="N113" s="13"/>
+      <c r="O113" s="13"/>
     </row>
     <row r="114">
       <c r="A114" s="13"/>
@@ -2055,6 +2174,7 @@
       <c r="L114" s="13"/>
       <c r="M114" s="13"/>
       <c r="N114" s="13"/>
+      <c r="O114" s="13"/>
     </row>
     <row r="115">
       <c r="A115" s="13"/>
@@ -2071,6 +2191,7 @@
       <c r="L115" s="13"/>
       <c r="M115" s="13"/>
       <c r="N115" s="13"/>
+      <c r="O115" s="13"/>
     </row>
     <row r="116">
       <c r="A116" s="13"/>
@@ -2087,6 +2208,7 @@
       <c r="L116" s="13"/>
       <c r="M116" s="13"/>
       <c r="N116" s="13"/>
+      <c r="O116" s="13"/>
     </row>
     <row r="117">
       <c r="A117" s="13"/>
@@ -2103,6 +2225,7 @@
       <c r="L117" s="13"/>
       <c r="M117" s="13"/>
       <c r="N117" s="13"/>
+      <c r="O117" s="13"/>
     </row>
     <row r="118">
       <c r="A118" s="13"/>
@@ -2119,6 +2242,7 @@
       <c r="L118" s="13"/>
       <c r="M118" s="13"/>
       <c r="N118" s="13"/>
+      <c r="O118" s="13"/>
     </row>
     <row r="119">
       <c r="A119" s="13"/>
@@ -2135,6 +2259,7 @@
       <c r="L119" s="13"/>
       <c r="M119" s="13"/>
       <c r="N119" s="13"/>
+      <c r="O119" s="13"/>
     </row>
     <row r="120">
       <c r="A120" s="13"/>
@@ -2151,6 +2276,7 @@
       <c r="L120" s="13"/>
       <c r="M120" s="13"/>
       <c r="N120" s="13"/>
+      <c r="O120" s="13"/>
     </row>
     <row r="121">
       <c r="A121" s="13"/>
@@ -2167,6 +2293,7 @@
       <c r="L121" s="13"/>
       <c r="M121" s="13"/>
       <c r="N121" s="13"/>
+      <c r="O121" s="13"/>
     </row>
     <row r="122">
       <c r="A122" s="13"/>
@@ -2183,6 +2310,7 @@
       <c r="L122" s="13"/>
       <c r="M122" s="13"/>
       <c r="N122" s="13"/>
+      <c r="O122" s="13"/>
     </row>
     <row r="123">
       <c r="A123" s="13"/>
@@ -2199,6 +2327,7 @@
       <c r="L123" s="13"/>
       <c r="M123" s="13"/>
       <c r="N123" s="13"/>
+      <c r="O123" s="13"/>
     </row>
     <row r="124">
       <c r="A124" s="13"/>
@@ -2215,6 +2344,7 @@
       <c r="L124" s="13"/>
       <c r="M124" s="13"/>
       <c r="N124" s="13"/>
+      <c r="O124" s="13"/>
     </row>
     <row r="125">
       <c r="A125" s="13"/>
@@ -2231,6 +2361,7 @@
       <c r="L125" s="13"/>
       <c r="M125" s="13"/>
       <c r="N125" s="13"/>
+      <c r="O125" s="13"/>
     </row>
     <row r="126">
       <c r="A126" s="13"/>
@@ -2247,6 +2378,7 @@
       <c r="L126" s="13"/>
       <c r="M126" s="13"/>
       <c r="N126" s="13"/>
+      <c r="O126" s="13"/>
     </row>
     <row r="127">
       <c r="A127" s="13"/>
@@ -2263,6 +2395,7 @@
       <c r="L127" s="13"/>
       <c r="M127" s="13"/>
       <c r="N127" s="13"/>
+      <c r="O127" s="13"/>
     </row>
     <row r="128">
       <c r="A128" s="13"/>
@@ -2279,6 +2412,7 @@
       <c r="L128" s="13"/>
       <c r="M128" s="13"/>
       <c r="N128" s="13"/>
+      <c r="O128" s="13"/>
     </row>
     <row r="129">
       <c r="A129" s="13"/>
@@ -2295,6 +2429,7 @@
       <c r="L129" s="13"/>
       <c r="M129" s="13"/>
       <c r="N129" s="13"/>
+      <c r="O129" s="13"/>
     </row>
     <row r="130">
       <c r="A130" s="13"/>
@@ -2311,6 +2446,7 @@
       <c r="L130" s="13"/>
       <c r="M130" s="13"/>
       <c r="N130" s="13"/>
+      <c r="O130" s="13"/>
     </row>
     <row r="131">
       <c r="A131" s="13"/>
@@ -2327,6 +2463,7 @@
       <c r="L131" s="13"/>
       <c r="M131" s="13"/>
       <c r="N131" s="13"/>
+      <c r="O131" s="13"/>
     </row>
     <row r="132">
       <c r="A132" s="13"/>
@@ -2343,6 +2480,7 @@
       <c r="L132" s="13"/>
       <c r="M132" s="13"/>
       <c r="N132" s="13"/>
+      <c r="O132" s="13"/>
     </row>
     <row r="133">
       <c r="A133" s="13"/>
@@ -2359,6 +2497,7 @@
       <c r="L133" s="13"/>
       <c r="M133" s="13"/>
       <c r="N133" s="13"/>
+      <c r="O133" s="13"/>
     </row>
     <row r="134">
       <c r="A134" s="13"/>
@@ -2375,6 +2514,7 @@
       <c r="L134" s="13"/>
       <c r="M134" s="13"/>
       <c r="N134" s="13"/>
+      <c r="O134" s="13"/>
     </row>
     <row r="135">
       <c r="A135" s="13"/>
@@ -2391,6 +2531,7 @@
       <c r="L135" s="13"/>
       <c r="M135" s="13"/>
       <c r="N135" s="13"/>
+      <c r="O135" s="13"/>
     </row>
     <row r="136">
       <c r="A136" s="13"/>
@@ -2407,6 +2548,7 @@
       <c r="L136" s="13"/>
       <c r="M136" s="13"/>
       <c r="N136" s="13"/>
+      <c r="O136" s="13"/>
     </row>
     <row r="137">
       <c r="A137" s="13"/>
@@ -2423,6 +2565,7 @@
       <c r="L137" s="13"/>
       <c r="M137" s="13"/>
       <c r="N137" s="13"/>
+      <c r="O137" s="13"/>
     </row>
     <row r="138">
       <c r="A138" s="13"/>
@@ -2439,6 +2582,7 @@
       <c r="L138" s="13"/>
       <c r="M138" s="13"/>
       <c r="N138" s="13"/>
+      <c r="O138" s="13"/>
     </row>
     <row r="139">
       <c r="A139" s="13"/>
@@ -2455,6 +2599,7 @@
       <c r="L139" s="13"/>
       <c r="M139" s="13"/>
       <c r="N139" s="13"/>
+      <c r="O139" s="13"/>
     </row>
     <row r="140">
       <c r="A140" s="13"/>
@@ -2471,6 +2616,7 @@
       <c r="L140" s="13"/>
       <c r="M140" s="13"/>
       <c r="N140" s="13"/>
+      <c r="O140" s="13"/>
     </row>
     <row r="141">
       <c r="A141" s="13"/>
@@ -2487,6 +2633,7 @@
       <c r="L141" s="13"/>
       <c r="M141" s="13"/>
       <c r="N141" s="13"/>
+      <c r="O141" s="13"/>
     </row>
     <row r="142">
       <c r="A142" s="13"/>
@@ -2503,6 +2650,7 @@
       <c r="L142" s="13"/>
       <c r="M142" s="13"/>
       <c r="N142" s="13"/>
+      <c r="O142" s="13"/>
     </row>
     <row r="143">
       <c r="A143" s="13"/>
@@ -2519,6 +2667,7 @@
       <c r="L143" s="13"/>
       <c r="M143" s="13"/>
       <c r="N143" s="13"/>
+      <c r="O143" s="13"/>
     </row>
     <row r="144">
       <c r="A144" s="13"/>
@@ -2535,6 +2684,7 @@
       <c r="L144" s="13"/>
       <c r="M144" s="13"/>
       <c r="N144" s="13"/>
+      <c r="O144" s="13"/>
     </row>
     <row r="145">
       <c r="A145" s="13"/>
@@ -2551,6 +2701,7 @@
       <c r="L145" s="13"/>
       <c r="M145" s="13"/>
       <c r="N145" s="13"/>
+      <c r="O145" s="13"/>
     </row>
     <row r="146">
       <c r="A146" s="13"/>
@@ -2567,6 +2718,7 @@
       <c r="L146" s="13"/>
       <c r="M146" s="13"/>
       <c r="N146" s="13"/>
+      <c r="O146" s="13"/>
     </row>
     <row r="147">
       <c r="A147" s="13"/>
@@ -2583,6 +2735,7 @@
       <c r="L147" s="13"/>
       <c r="M147" s="13"/>
       <c r="N147" s="13"/>
+      <c r="O147" s="13"/>
     </row>
     <row r="148">
       <c r="A148" s="13"/>
@@ -2599,6 +2752,7 @@
       <c r="L148" s="13"/>
       <c r="M148" s="13"/>
       <c r="N148" s="13"/>
+      <c r="O148" s="13"/>
     </row>
     <row r="149">
       <c r="A149" s="13"/>
@@ -2615,6 +2769,7 @@
       <c r="L149" s="13"/>
       <c r="M149" s="13"/>
       <c r="N149" s="13"/>
+      <c r="O149" s="13"/>
     </row>
     <row r="150">
       <c r="A150" s="13"/>
@@ -2631,6 +2786,7 @@
       <c r="L150" s="13"/>
       <c r="M150" s="13"/>
       <c r="N150" s="13"/>
+      <c r="O150" s="13"/>
     </row>
     <row r="151">
       <c r="A151" s="13"/>
@@ -2647,6 +2803,7 @@
       <c r="L151" s="13"/>
       <c r="M151" s="13"/>
       <c r="N151" s="13"/>
+      <c r="O151" s="13"/>
     </row>
     <row r="152">
       <c r="A152" s="13"/>
@@ -2663,6 +2820,7 @@
       <c r="L152" s="13"/>
       <c r="M152" s="13"/>
       <c r="N152" s="13"/>
+      <c r="O152" s="13"/>
     </row>
     <row r="153">
       <c r="A153" s="13"/>
@@ -2679,6 +2837,7 @@
       <c r="L153" s="13"/>
       <c r="M153" s="13"/>
       <c r="N153" s="13"/>
+      <c r="O153" s="13"/>
     </row>
     <row r="154">
       <c r="A154" s="13"/>
@@ -2695,6 +2854,7 @@
       <c r="L154" s="13"/>
       <c r="M154" s="13"/>
       <c r="N154" s="13"/>
+      <c r="O154" s="13"/>
     </row>
     <row r="155">
       <c r="A155" s="13"/>
@@ -2711,6 +2871,7 @@
       <c r="L155" s="13"/>
       <c r="M155" s="13"/>
       <c r="N155" s="13"/>
+      <c r="O155" s="13"/>
     </row>
     <row r="156">
       <c r="A156" s="13"/>
@@ -2727,6 +2888,7 @@
       <c r="L156" s="13"/>
       <c r="M156" s="13"/>
       <c r="N156" s="13"/>
+      <c r="O156" s="13"/>
     </row>
     <row r="157">
       <c r="A157" s="13"/>
@@ -2743,6 +2905,7 @@
       <c r="L157" s="13"/>
       <c r="M157" s="13"/>
       <c r="N157" s="13"/>
+      <c r="O157" s="13"/>
     </row>
     <row r="158">
       <c r="A158" s="13"/>
@@ -2759,6 +2922,7 @@
       <c r="L158" s="13"/>
       <c r="M158" s="13"/>
       <c r="N158" s="13"/>
+      <c r="O158" s="13"/>
     </row>
     <row r="159">
       <c r="A159" s="13"/>
@@ -2775,6 +2939,7 @@
       <c r="L159" s="13"/>
       <c r="M159" s="13"/>
       <c r="N159" s="13"/>
+      <c r="O159" s="13"/>
     </row>
     <row r="160">
       <c r="A160" s="13"/>
@@ -2791,6 +2956,7 @@
       <c r="L160" s="13"/>
       <c r="M160" s="13"/>
       <c r="N160" s="13"/>
+      <c r="O160" s="13"/>
     </row>
     <row r="161">
       <c r="A161" s="13"/>
@@ -2807,6 +2973,7 @@
       <c r="L161" s="13"/>
       <c r="M161" s="13"/>
       <c r="N161" s="13"/>
+      <c r="O161" s="13"/>
     </row>
     <row r="162">
       <c r="A162" s="13"/>
@@ -2823,6 +2990,7 @@
       <c r="L162" s="13"/>
       <c r="M162" s="13"/>
       <c r="N162" s="13"/>
+      <c r="O162" s="13"/>
     </row>
     <row r="163">
       <c r="A163" s="13"/>
@@ -2839,6 +3007,7 @@
       <c r="L163" s="13"/>
       <c r="M163" s="13"/>
       <c r="N163" s="13"/>
+      <c r="O163" s="13"/>
     </row>
     <row r="164">
       <c r="A164" s="13"/>
@@ -2855,6 +3024,7 @@
       <c r="L164" s="13"/>
       <c r="M164" s="13"/>
       <c r="N164" s="13"/>
+      <c r="O164" s="13"/>
     </row>
     <row r="165">
       <c r="A165" s="13"/>
@@ -2871,6 +3041,7 @@
       <c r="L165" s="13"/>
       <c r="M165" s="13"/>
       <c r="N165" s="13"/>
+      <c r="O165" s="13"/>
     </row>
     <row r="166">
       <c r="A166" s="13"/>
@@ -2887,6 +3058,7 @@
       <c r="L166" s="13"/>
       <c r="M166" s="13"/>
       <c r="N166" s="13"/>
+      <c r="O166" s="13"/>
     </row>
     <row r="167">
       <c r="A167" s="13"/>
@@ -2903,6 +3075,7 @@
       <c r="L167" s="13"/>
       <c r="M167" s="13"/>
       <c r="N167" s="13"/>
+      <c r="O167" s="13"/>
     </row>
     <row r="168">
       <c r="A168" s="13"/>
@@ -2919,6 +3092,7 @@
       <c r="L168" s="13"/>
       <c r="M168" s="13"/>
       <c r="N168" s="13"/>
+      <c r="O168" s="13"/>
     </row>
     <row r="169">
       <c r="A169" s="13"/>
@@ -2935,6 +3109,7 @@
       <c r="L169" s="13"/>
       <c r="M169" s="13"/>
       <c r="N169" s="13"/>
+      <c r="O169" s="13"/>
     </row>
     <row r="170">
       <c r="A170" s="13"/>
@@ -2951,6 +3126,7 @@
       <c r="L170" s="13"/>
       <c r="M170" s="13"/>
       <c r="N170" s="13"/>
+      <c r="O170" s="13"/>
     </row>
     <row r="171">
       <c r="A171" s="13"/>
@@ -2967,6 +3143,7 @@
       <c r="L171" s="13"/>
       <c r="M171" s="13"/>
       <c r="N171" s="13"/>
+      <c r="O171" s="13"/>
     </row>
     <row r="172">
       <c r="A172" s="13"/>
@@ -2983,6 +3160,7 @@
       <c r="L172" s="13"/>
       <c r="M172" s="13"/>
       <c r="N172" s="13"/>
+      <c r="O172" s="13"/>
     </row>
     <row r="173">
       <c r="A173" s="13"/>
@@ -2999,6 +3177,7 @@
       <c r="L173" s="13"/>
       <c r="M173" s="13"/>
       <c r="N173" s="13"/>
+      <c r="O173" s="13"/>
     </row>
     <row r="174">
       <c r="A174" s="13"/>
@@ -3015,6 +3194,7 @@
       <c r="L174" s="13"/>
       <c r="M174" s="13"/>
       <c r="N174" s="13"/>
+      <c r="O174" s="13"/>
     </row>
     <row r="175">
       <c r="A175" s="13"/>
@@ -3031,6 +3211,7 @@
       <c r="L175" s="13"/>
       <c r="M175" s="13"/>
       <c r="N175" s="13"/>
+      <c r="O175" s="13"/>
     </row>
     <row r="176">
       <c r="A176" s="13"/>
@@ -3047,6 +3228,7 @@
       <c r="L176" s="13"/>
       <c r="M176" s="13"/>
       <c r="N176" s="13"/>
+      <c r="O176" s="13"/>
     </row>
     <row r="177">
       <c r="A177" s="13"/>
@@ -3063,6 +3245,7 @@
       <c r="L177" s="13"/>
       <c r="M177" s="13"/>
       <c r="N177" s="13"/>
+      <c r="O177" s="13"/>
     </row>
     <row r="178">
       <c r="A178" s="13"/>
@@ -3079,6 +3262,7 @@
       <c r="L178" s="13"/>
       <c r="M178" s="13"/>
       <c r="N178" s="13"/>
+      <c r="O178" s="13"/>
     </row>
     <row r="179">
       <c r="A179" s="13"/>
@@ -3095,6 +3279,7 @@
       <c r="L179" s="13"/>
       <c r="M179" s="13"/>
       <c r="N179" s="13"/>
+      <c r="O179" s="13"/>
     </row>
     <row r="180">
       <c r="A180" s="13"/>
@@ -3111,6 +3296,7 @@
       <c r="L180" s="13"/>
       <c r="M180" s="13"/>
       <c r="N180" s="13"/>
+      <c r="O180" s="13"/>
     </row>
     <row r="181">
       <c r="A181" s="13"/>
@@ -3127,6 +3313,7 @@
       <c r="L181" s="13"/>
       <c r="M181" s="13"/>
       <c r="N181" s="13"/>
+      <c r="O181" s="13"/>
     </row>
     <row r="182">
       <c r="A182" s="13"/>
@@ -3143,6 +3330,7 @@
       <c r="L182" s="13"/>
       <c r="M182" s="13"/>
       <c r="N182" s="13"/>
+      <c r="O182" s="13"/>
     </row>
     <row r="183">
       <c r="A183" s="13"/>
@@ -3159,6 +3347,7 @@
       <c r="L183" s="13"/>
       <c r="M183" s="13"/>
       <c r="N183" s="13"/>
+      <c r="O183" s="13"/>
     </row>
     <row r="184">
       <c r="A184" s="13"/>
@@ -3175,6 +3364,7 @@
       <c r="L184" s="13"/>
       <c r="M184" s="13"/>
       <c r="N184" s="13"/>
+      <c r="O184" s="13"/>
     </row>
     <row r="185">
       <c r="A185" s="13"/>
@@ -3191,6 +3381,7 @@
       <c r="L185" s="13"/>
       <c r="M185" s="13"/>
       <c r="N185" s="13"/>
+      <c r="O185" s="13"/>
     </row>
     <row r="186">
       <c r="A186" s="13"/>
@@ -3207,6 +3398,7 @@
       <c r="L186" s="13"/>
       <c r="M186" s="13"/>
       <c r="N186" s="13"/>
+      <c r="O186" s="13"/>
     </row>
     <row r="187">
       <c r="A187" s="13"/>
@@ -3223,6 +3415,7 @@
       <c r="L187" s="13"/>
       <c r="M187" s="13"/>
       <c r="N187" s="13"/>
+      <c r="O187" s="13"/>
     </row>
     <row r="188">
       <c r="A188" s="13"/>
@@ -3239,6 +3432,7 @@
       <c r="L188" s="13"/>
       <c r="M188" s="13"/>
       <c r="N188" s="13"/>
+      <c r="O188" s="13"/>
     </row>
     <row r="189">
       <c r="A189" s="13"/>
@@ -3255,6 +3449,7 @@
       <c r="L189" s="13"/>
       <c r="M189" s="13"/>
       <c r="N189" s="13"/>
+      <c r="O189" s="13"/>
     </row>
     <row r="190">
       <c r="A190" s="13"/>
@@ -3271,6 +3466,7 @@
       <c r="L190" s="13"/>
       <c r="M190" s="13"/>
       <c r="N190" s="13"/>
+      <c r="O190" s="13"/>
     </row>
     <row r="191">
       <c r="A191" s="13"/>
@@ -3287,6 +3483,7 @@
       <c r="L191" s="13"/>
       <c r="M191" s="13"/>
       <c r="N191" s="13"/>
+      <c r="O191" s="13"/>
     </row>
     <row r="192">
       <c r="A192" s="13"/>
@@ -3303,6 +3500,7 @@
       <c r="L192" s="13"/>
       <c r="M192" s="13"/>
       <c r="N192" s="13"/>
+      <c r="O192" s="13"/>
     </row>
     <row r="193">
       <c r="A193" s="13"/>
@@ -3319,6 +3517,7 @@
       <c r="L193" s="13"/>
       <c r="M193" s="13"/>
       <c r="N193" s="13"/>
+      <c r="O193" s="13"/>
     </row>
     <row r="194">
       <c r="A194" s="13"/>
@@ -3335,6 +3534,7 @@
       <c r="L194" s="13"/>
       <c r="M194" s="13"/>
       <c r="N194" s="13"/>
+      <c r="O194" s="13"/>
     </row>
     <row r="195">
       <c r="A195" s="13"/>
@@ -3351,6 +3551,7 @@
       <c r="L195" s="13"/>
       <c r="M195" s="13"/>
       <c r="N195" s="13"/>
+      <c r="O195" s="13"/>
     </row>
     <row r="196">
       <c r="A196" s="13"/>
@@ -3367,6 +3568,7 @@
       <c r="L196" s="13"/>
       <c r="M196" s="13"/>
       <c r="N196" s="13"/>
+      <c r="O196" s="13"/>
     </row>
     <row r="197">
       <c r="A197" s="13"/>
@@ -3383,6 +3585,7 @@
       <c r="L197" s="13"/>
       <c r="M197" s="13"/>
       <c r="N197" s="13"/>
+      <c r="O197" s="13"/>
     </row>
     <row r="198">
       <c r="A198" s="13"/>
@@ -3399,6 +3602,7 @@
       <c r="L198" s="13"/>
       <c r="M198" s="13"/>
       <c r="N198" s="13"/>
+      <c r="O198" s="13"/>
     </row>
     <row r="199">
       <c r="A199" s="13"/>
@@ -3415,6 +3619,7 @@
       <c r="L199" s="13"/>
       <c r="M199" s="13"/>
       <c r="N199" s="13"/>
+      <c r="O199" s="13"/>
     </row>
     <row r="200">
       <c r="A200" s="13"/>
@@ -3431,6 +3636,7 @@
       <c r="L200" s="13"/>
       <c r="M200" s="13"/>
       <c r="N200" s="13"/>
+      <c r="O200" s="13"/>
     </row>
     <row r="201">
       <c r="A201" s="13"/>
@@ -3447,9 +3653,10 @@
       <c r="L201" s="13"/>
       <c r="M201" s="13"/>
       <c r="N201" s="13"/>
+      <c r="O201" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N5001"/>
+  <autoFilter ref="A1:O5001"/>
   <dataValidations count="5">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="每个SKU一个唯一编号，宝可梦PK-前缀，符文战场RB-前缀；不同单位分别编号。" errorTitle="请检查输入" error="编号已重复。" sqref="A2:A5001">
       <formula1>COUNTIF($A$2:$A$5001,A2)=1</formula1>
@@ -3457,13 +3664,13 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="选择补充包、周边或礼盒·预组。" errorTitle="请检查输入" error="请选择补充包、周边或礼盒·预组。" sqref="C2:C5001">
       <formula1>"补充包,周边,礼盒·预组"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="肥包、瘦包或留空；包规格在J列自由填写。" errorTitle="请检查输入" error="请选择肥包、瘦包或留空。" sqref="K2:K5001">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="肥包、瘦包或留空；包规格在K列自由填写。" errorTitle="请检查输入" error="请选择肥包、瘦包或留空。" sqref="L2:L5001">
       <formula1>"肥包,瘦包"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="仅作包装说明，例如20盒/箱、6张/包，不自动换算。" errorTitle="请检查输入" error="请填写规格说明。" sqref="I2:J5001">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="仅作包装说明，例如20中盒/箱、18包/中盒、4张/包，不自动换算。" errorTitle="请检查输入" error="请填写规格说明。" sqref="I2:K5001">
       <formula1>TRUE</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="多个别名用中文分号“；”分隔。" errorTitle="请检查输入" error="请按说明填写。" sqref="F2:F5001 N2:N5001">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" promptTitle="填写提示" prompt="多个别名用中文分号“；”分隔。" errorTitle="请检查输入" error="请按说明填写。" sqref="F2:F5001 O2:O5001">
       <formula1>TRUE</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>